<commit_message>
Add initial Excel file and create start-dev.bat script for development setup
</commit_message>
<xml_diff>
--- a/Thursday Reschedule.xlsx
+++ b/Thursday Reschedule.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f80e6e0943a1a34c/Desktop/Email Tool/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f80e6e0943a1a34c/Desktop/Old Email Tool/Email_Tool/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="11_79C3E2171C397D6A206102A720D19643A12CC1D0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7EC84672-F517-4A19-8A31-1AD1958F6D6D}"/>
+  <xr:revisionPtr revIDLastSave="40" documentId="11_79C3E2171C397D6A206102A720D19643A12CC1D0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46C61CAB-1442-4326-9E66-F618F7B3DFC2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="82">
   <si>
     <t>company</t>
   </si>
@@ -35,15 +35,6 @@
     <t>schedule</t>
   </si>
   <si>
-    <t>Software Engineer</t>
-  </si>
-  <si>
-    <t>Trusted</t>
-  </si>
-  <si>
-    <t>anup.anything@yahoo.com, anuppofficial.002@gmail.com</t>
-  </si>
-  <si>
     <t>rutuja.bhailume@zoop.one, hr@zoop.one</t>
   </si>
   <si>
@@ -218,67 +209,64 @@
     <t>Zoop</t>
   </si>
   <si>
-    <t>Thu 09:00</t>
-  </si>
-  <si>
-    <t>Thu 09:01</t>
-  </si>
-  <si>
-    <t>Thu 09:02</t>
-  </si>
-  <si>
-    <t>Thu 09:03</t>
-  </si>
-  <si>
-    <t>Thu 09:04</t>
-  </si>
-  <si>
-    <t>Thu 09:05</t>
-  </si>
-  <si>
-    <t>Thu 09:06</t>
-  </si>
-  <si>
-    <t>Thu 09:07</t>
-  </si>
-  <si>
-    <t>Thu 09:08</t>
-  </si>
-  <si>
-    <t>Thu 09:09</t>
-  </si>
-  <si>
-    <t>Thu 09:10</t>
-  </si>
-  <si>
-    <t>Thu 09:11</t>
-  </si>
-  <si>
-    <t>Thu 09:12</t>
-  </si>
-  <si>
-    <t>Thu 09:13</t>
-  </si>
-  <si>
-    <t>Thu 09:14</t>
-  </si>
-  <si>
-    <t>Thu 09:15</t>
-  </si>
-  <si>
-    <t>Thu 09:16</t>
-  </si>
-  <si>
-    <t>Thu 09:17</t>
-  </si>
-  <si>
-    <t>Thu 09:18</t>
-  </si>
-  <si>
-    <t>Thu 09:19</t>
-  </si>
-  <si>
-    <t>Thu 09:20</t>
+    <t>Thu,Mon 09:01</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:02</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:03</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:04</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:05</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:06</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:07</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:08</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:09</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:10</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:11</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:12</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:13</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:14</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:15</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:16</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:17</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:18</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:19</t>
+  </si>
+  <si>
+    <t>Thu,Mon 09:20</t>
   </si>
 </sst>
 </file>
@@ -751,7 +739,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.25" style="3" customWidth="1"/>
@@ -775,36 +763,37 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="D2" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="8" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>66</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="E3" s="9"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
@@ -813,11 +802,11 @@
       <c r="B4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="6" t="s">
         <v>11</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="E4" s="9"/>
     </row>
@@ -825,208 +814,207 @@
       <c r="A5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E5" s="9"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="4" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>17</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E6" s="9"/>
     </row>
-    <row r="7" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="E7" s="9"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>22</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>23</v>
       </c>
       <c r="C8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="B9" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="C11" s="6" t="s">
+      <c r="E11" s="12" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>31</v>
-      </c>
-      <c r="B12" t="s">
-        <v>58</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>32</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="75" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>35</v>
+      <c r="C13" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="C14" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="D14" s="1" t="s">
+      <c r="B15" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E15">
+        <v>9203400170</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D17" s="1" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D15" s="1" t="s">
+    <row r="18" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="B16" t="s">
-        <v>60</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="E16">
-        <v>9203400170</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>45</v>
       </c>
@@ -1037,59 +1025,45 @@
         <v>47</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>48</v>
       </c>
       <c r="B20" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="6" t="s">
         <v>50</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="13" t="s">
         <v>51</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="B11" r:id="rId1" xr:uid="{5B5772F8-F6BE-482D-9E90-8AB998B6CFE0}"/>
+    <hyperlink ref="B10" r:id="rId1" xr:uid="{5B5772F8-F6BE-482D-9E90-8AB998B6CFE0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="B1:D1 C2" numberStoredAsText="1"/>
+    <ignoredError sqref="B1:D1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1101,11 +1075,11 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="10" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D1" s="11"/>
       <c r="E1" s="12">

</xml_diff>